<commit_message>
Remove internal research notes from public edition
</commit_message>
<xml_diff>
--- a/Paterson Giving Map - Donor Database.xlsx
+++ b/Paterson Giving Map - Donor Database.xlsx
@@ -929,7 +929,7 @@
       </c>
       <c r="J3" s="13" t="inlineStr">
         <is>
-          <t>Largest documented private family funder of Paterson human services in 2023-2025 (approx. $2.7M to Eva's Village and St. Joseph's in three tax years). Foundation assets ~$7.8M (FY2025). Lifetime 'Over $1 Million' donor to St. Joseph's Health Foundation. Foundation states it funds only preselected organizations. Family members Anthony M. LoConte and Gabriella LoConte also appear individually on St. Joseph's honor rolls.</t>
+          <t>Anthony M. LoConte, President &amp; CEO, Anthony L &amp; S LLC (shoe importer/distributor); Hudson County real estate developer</t>
         </is>
       </c>
       <c r="K3" s="10" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>$15M-asset foundation, ~$1M/yr distributions, Passaic County focus (also $500K Passaic HS scholarship program 2026 and William Paterson University library gift 2023). St. Joseph's is Paterson-based; the named lobby is at the Totowa campus.</t>
+          <t>William J. Martini - U.S. District Judge (D.N.J.), former Congressman; foundation founded 1986 by former Passaic Mayor Nicholas Martini</t>
         </is>
       </c>
       <c r="K10" s="10" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="J21" s="13" t="inlineStr">
         <is>
-          <t>Paterson-headquartered family foundation ($3.8M assets, $500K contributed in FY2025). Railroad Construction Co. also appears at $50K-$99K on SJHF rolls and was honored by Paterson Habitat (2022). Company also an NJCDC 'Above and Beyond' donor (2026). One of the most Paterson-concentrated private donors identified.</t>
+          <t>Century-old Paterson company (est. 1926); Title Sponsor of Eva's Village 2025 gala and 2026 gala honoree; NRTC contributor (as RCC Builders &amp; Developers) to NJCDC and Paterson Habitat FY2021; honored by Paterson Habitat 2022; longtime Boys &amp; Girls Club partner. EVP Daniel Cipoletti is Eva's Village board vice chair; CEO Al Daloisio Jr. on Eva's board.</t>
         </is>
       </c>
       <c r="K21" s="10" t="inlineStr">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="J33" s="13" t="inlineStr">
         <is>
-          <t>Planned-gift example; no living prospect.</t>
+          <t>Bequest</t>
         </is>
       </c>
       <c r="K33" s="10" t="inlineStr"/>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="J37" s="13" t="inlineStr">
         <is>
-          <t>Planned-gift example; no living prospect.</t>
+          <t>Bequest</t>
         </is>
       </c>
       <c r="K37" s="10" t="inlineStr"/>
@@ -3375,7 +3375,7 @@
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>Consistent five/six-figure annual support; trust structure means living family involvement is unclear.</t>
+          <t>Charitable trust named for Richard J. and Mary F. Walsh</t>
         </is>
       </c>
       <c r="K40" s="10" t="inlineStr">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="J42" s="13" t="inlineStr">
         <is>
-          <t>Physician-donor couple; Moira Connolly serves on SJHF board and gala committees.</t>
+          <t>Mark Connolly, MD - cardiothoracic surgeon, St. Joseph's University Medical Center, Paterson; Moira Connolly - Principal, M K Connolly LLC (healthcare risk consulting); SJHF trustee</t>
         </is>
       </c>
       <c r="K42" s="10" t="inlineStr"/>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>Six-figure annual donor to Paterson's hospital; professional affiliation not found in public sources.</t>
+          <t>Not publicly reported</t>
         </is>
       </c>
       <c r="K49" s="10" t="inlineStr"/>
@@ -4049,7 +4049,7 @@
       </c>
       <c r="J51" s="13" t="inlineStr">
         <is>
-          <t>20+ years of St. Joseph's governance; affiliation per https://www.citrincooperman.com/In-Focus-Resource-Center/Wilfredo-Fernandez-receives-the-Robert-M-Marcalus-Legacy-Award.</t>
+          <t>Wilfredo Fernandez - Partner, Citrin Cooperman; Chair, St. Joseph's Health Board (2020-2024/25); Robert L. Marcalus Legacy Award 2025</t>
         </is>
       </c>
       <c r="K51" s="10" t="inlineStr"/>
@@ -4239,7 +4239,7 @@
       </c>
       <c r="J54" s="13" t="inlineStr">
         <is>
-          <t>Consistent $50K+/yr donor; listed on 2019 and 2020 rolls as well.</t>
+          <t>Not publicly reported (Charles Breuss deceased)</t>
         </is>
       </c>
       <c r="K54" s="10" t="inlineStr"/>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>Executive-donor; gala honoree 2023 (https://givetostjosephs.org/events/gala2023/).</t>
+          <t>Kevin J. Slavin - President &amp; CEO, St. Joseph's Health (Paterson) through 2025; Robert L. Marcalus Legacy Award 2023</t>
         </is>
       </c>
       <c r="K55" s="10" t="inlineStr"/>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>Paterson business owner giving primarily through the company.</t>
+          <t>President &amp; CEO, Reno's Appliance Inc. (Paterson); SJHF trustee; 2024 Robert L. Marcalus Legacy Award</t>
         </is>
       </c>
       <c r="K57" s="10" t="inlineStr">
@@ -4475,7 +4475,7 @@
       </c>
       <c r="J58" s="13" t="inlineStr">
         <is>
-          <t>Board chair-level volunteer and donor. Affiliation per https://givetostjosephs.org/about/board-of-trustees/.</t>
+          <t>Dean P. Emmolo - President, Faber Industrial Technologies; Chair, St. Joseph's Health Foundation Board of Trustees (2021-2023); 2025 Gala co-chairs</t>
         </is>
       </c>
       <c r="K58" s="10" t="inlineStr"/>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="J63" s="13" t="inlineStr">
         <is>
-          <t>Catholic-oriented Bergen County family foundation; Eva's Village is among its largest grantees ($50K-$70K/yr).</t>
+          <t>Not publicly reported</t>
         </is>
       </c>
       <c r="K63" s="10" t="inlineStr">
@@ -4837,7 +4837,7 @@
       </c>
       <c r="J64" s="13" t="inlineStr">
         <is>
-          <t>Below $25K threshold but a named, recurring Paterson scholarship fund.</t>
+          <t>Not publicly reported</t>
         </is>
       </c>
       <c r="K64" s="10" t="inlineStr"/>
@@ -5147,7 +5147,7 @@
       </c>
       <c r="J69" s="13" t="inlineStr">
         <is>
-          <t>Physician-donor; gives personally and through practice.</t>
+          <t>Arash Emami, MD - spine surgeon, University Spine Center (Wayne); St. Joseph's medical staff</t>
         </is>
       </c>
       <c r="K69" s="10" t="inlineStr"/>
@@ -5499,7 +5499,7 @@
       </c>
       <c r="J75" s="13" t="inlineStr">
         <is>
-          <t>Paterson employer (~90% of workforce are Paterson residents); received Greater Paterson Chamber 'Faith in Paterson' award. Nancy Kontos chairs SJHF board (https://givetostjosephs.org/about/board-of-trustees/).</t>
+          <t>Steve Kontos - Vice President, Kontos Foods Inc. (Paterson-based Mediterranean foods manufacturer); Nancy Kontos - CFO, Kontos Foods and Chair, St. Joseph's Health Foundation Board</t>
         </is>
       </c>
       <c r="K75" s="10" t="inlineStr">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="J82" s="13" t="inlineStr">
         <is>
-          <t>Affiliation inferred from public bio; verify before use.</t>
+          <t>Higher-education executive (former Executive Vice President, Seton Hall University; interim president)</t>
         </is>
       </c>
       <c r="K82" s="10" t="inlineStr"/>
@@ -5957,7 +5957,7 @@
       </c>
       <c r="J83" s="13" t="inlineStr">
         <is>
-          <t>Personal plus company giving to Paterson hospital.</t>
+          <t>Joseph Amico - VP/Owner, EVS Metal (Riverdale, NJ); SJHF trustee</t>
         </is>
       </c>
       <c r="K83" s="10" t="inlineStr"/>
@@ -6081,7 +6081,7 @@
       </c>
       <c r="J85" s="13" t="inlineStr">
         <is>
-          <t>German-American heritage foundation; Oasis is a consistent top-3 grantee.</t>
+          <t>Not publicly reported; 'Mr. and Mrs. Joseph Pfeifer' also on St. Joseph's Health Foundation lifetime $250,000-$499,999 honor roll</t>
         </is>
       </c>
       <c r="K85" s="10" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="J89" s="13" t="inlineStr">
         <is>
-          <t>Physician-donor couple profiled in 2021 impact report.</t>
+          <t>Roberto Solis, MD - physician, St. Joseph's Health (featured donor interview 2021)</t>
         </is>
       </c>
       <c r="K89" s="10" t="inlineStr"/>
@@ -6515,7 +6515,7 @@
       </c>
       <c r="J92" s="13" t="inlineStr">
         <is>
-          <t>One of the few identifiable family-foundation donors to Hamilton Partnership; NYC-based, arts/education focus.</t>
+          <t>James D. Krugman - attorney; Candace K. Beinecke - Senior Partner, Hughes Hubbard &amp; Reed</t>
         </is>
       </c>
       <c r="K92" s="10" t="inlineStr">
@@ -6769,7 +6769,7 @@
       </c>
       <c r="J96" s="13" t="inlineStr">
         <is>
-          <t>Physician-donor.</t>
+          <t>Mahesh Bikkina, MD - Chief of Cardiology, St. Joseph's University Medical Center</t>
         </is>
       </c>
       <c r="K96" s="10" t="inlineStr"/>
@@ -6823,7 +6823,7 @@
       </c>
       <c r="J97" s="13" t="inlineStr">
         <is>
-          <t>Recurring, growing gifts to Paterson hospital from a NYC family foundation.</t>
+          <t>Not publicly reported</t>
         </is>
       </c>
       <c r="K97" s="10" t="inlineStr">
@@ -48857,7 +48857,7 @@
       </c>
       <c r="J7" s="13" t="inlineStr">
         <is>
-          <t>Executive-donor; has since left the region (Nemours, Wilmington DE).</t>
+          <t>Caswell L. Samms III - SVP &amp; CFO, St. Joseph's Health (Dec 2020-2025); now EVP/CFO, Nemours Children's Health</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr"/>
@@ -49039,7 +49039,7 @@
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>2025 gala honoree (https://givetostjosephs.org/events/gala2025/).</t>
+          <t>Hillel Ephros, DMD, MD - Chairman, Dentistry/Oral &amp; Maxillofacial Surgery, St. Joseph's Health; 2025 Kendrick P. Lance Distinguished Physician Award</t>
         </is>
       </c>
       <c r="K10" s="10" t="inlineStr"/>
@@ -49093,7 +49093,7 @@
       </c>
       <c r="J11" s="13" t="inlineStr">
         <is>
-          <t>2023 gala honoree.</t>
+          <t>Roger Kierce, MD - Chair, Obstetrics and Gynecology, St. Joseph's Health; 2023 Kendrick P. Lance Distinguished Physician Award</t>
         </is>
       </c>
       <c r="K11" s="10" t="inlineStr"/>
@@ -49197,7 +49197,7 @@
       </c>
       <c r="J13" s="13" t="inlineStr">
         <is>
-          <t>Board member with quarter-million-plus lifetime giving.</t>
+          <t>Real estate investor, Olirei Investments LLC; SJHF trustee</t>
         </is>
       </c>
       <c r="K13" s="10" t="inlineStr"/>
@@ -50293,7 +50293,7 @@
       </c>
       <c r="J31" s="13" t="inlineStr">
         <is>
-          <t>Likely memorial giving.</t>
+          <t>Not publicly reported (Charles Cohen deceased)</t>
         </is>
       </c>
       <c r="K31" s="10" t="inlineStr"/>
@@ -51097,7 +51097,7 @@
       </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>Deceased; possible estate/family follow-up only.</t>
+          <t>Not publicly reported (deceased)</t>
         </is>
       </c>
       <c r="K44" s="10" t="inlineStr"/>
@@ -51151,7 +51151,7 @@
       </c>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>Seven-figure lifetime physician-donor.</t>
+          <t>James LaBagnara, MD - otolaryngologist, St. Joseph's medical staff (Paterson)</t>
         </is>
       </c>
       <c r="K45" s="10" t="inlineStr"/>

</xml_diff>